<commit_message>
Updating the model for Adrem
</commit_message>
<xml_diff>
--- a/data_fetching/Entsoe/Actual_Production_Solar.xlsx
+++ b/data_fetching/Entsoe/Actual_Production_Solar.xlsx
@@ -394,7 +394,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2">
-        <v>46146.01041666666</v>
+        <v>46148.01041666666</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -402,7 +402,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2">
-        <v>46146.02083333334</v>
+        <v>46148.02083333334</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -410,7 +410,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2">
-        <v>46146.03125</v>
+        <v>46148.03125</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -418,7 +418,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2">
-        <v>46146.04166666666</v>
+        <v>46148.04166666666</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -426,7 +426,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2">
-        <v>46146.05208333334</v>
+        <v>46148.05208333334</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -434,7 +434,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2">
-        <v>46146.0625</v>
+        <v>46148.0625</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -442,7 +442,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2">
-        <v>46146.07291666666</v>
+        <v>46148.07291666666</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -450,7 +450,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2">
-        <v>46146.08333333334</v>
+        <v>46148.08333333334</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -458,7 +458,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2">
-        <v>46146.09375</v>
+        <v>46148.09375</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -466,7 +466,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2">
-        <v>46146.10416666666</v>
+        <v>46148.10416666666</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -474,7 +474,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2">
-        <v>46146.11458333334</v>
+        <v>46148.11458333334</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -482,7 +482,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2">
-        <v>46146.125</v>
+        <v>46148.125</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -490,7 +490,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2">
-        <v>46146.13541666666</v>
+        <v>46148.13541666666</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -498,7 +498,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2">
-        <v>46146.14583333334</v>
+        <v>46148.14583333334</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -506,7 +506,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2">
-        <v>46146.15625</v>
+        <v>46148.15625</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -514,7 +514,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2">
-        <v>46146.16666666666</v>
+        <v>46148.16666666666</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -522,7 +522,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2">
-        <v>46146.17708333334</v>
+        <v>46148.17708333334</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -530,7 +530,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2">
-        <v>46146.1875</v>
+        <v>46148.1875</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -538,7 +538,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2">
-        <v>46146.19791666666</v>
+        <v>46148.19791666666</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -546,7 +546,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2">
-        <v>46146.20833333334</v>
+        <v>46148.20833333334</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -554,7 +554,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="2">
-        <v>46146.21875</v>
+        <v>46148.21875</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -562,119 +562,119 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="2">
-        <v>46146.22916666666</v>
+        <v>46148.22916666666</v>
       </c>
       <c r="B23">
-        <v>8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="2">
-        <v>46146.23958333334</v>
+        <v>46148.23958333334</v>
       </c>
       <c r="B24">
-        <v>46</v>
+        <v>60</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="2">
-        <v>46146.25</v>
+        <v>46148.25</v>
       </c>
       <c r="B25">
-        <v>93</v>
+        <v>124</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2">
-        <v>46146.26041666666</v>
+        <v>46148.26041666666</v>
       </c>
       <c r="B26">
-        <v>188</v>
+        <v>211</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="2">
-        <v>46146.27083333334</v>
+        <v>46148.27083333334</v>
       </c>
       <c r="B27">
-        <v>312</v>
+        <v>334</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="2">
-        <v>46146.28125</v>
+        <v>46148.28125</v>
       </c>
       <c r="B28">
-        <v>459</v>
+        <v>469</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="2">
-        <v>46146.29166666666</v>
+        <v>46148.29166666666</v>
       </c>
       <c r="B29">
-        <v>595</v>
+        <v>629</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="2">
-        <v>46146.30208333334</v>
+        <v>46148.30208333334</v>
       </c>
       <c r="B30">
-        <v>824</v>
+        <v>786</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="2">
-        <v>46146.3125</v>
+        <v>46148.3125</v>
       </c>
       <c r="B31">
-        <v>1011</v>
+        <v>992</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="2">
-        <v>46146.32291666666</v>
+        <v>46148.32291666666</v>
       </c>
       <c r="B32">
-        <v>1168</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="2">
-        <v>46146.33333333334</v>
+        <v>46148.33333333334</v>
       </c>
       <c r="B33">
-        <v>1322</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="2">
-        <v>46146.34375</v>
+        <v>46148.34375</v>
       </c>
       <c r="B34">
-        <v>1450</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="2">
-        <v>46146.35416666666</v>
+        <v>46148.35416666666</v>
       </c>
       <c r="B35">
-        <v>1576</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="2">
-        <v>46146.36458333334</v>
+        <v>46148.36458333334</v>
       </c>
       <c r="B36">
-        <v>1728</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="2">
-        <v>46146.375</v>
+        <v>46148.375</v>
       </c>
       <c r="B37">
         <v>0</v>
@@ -682,7 +682,7 @@
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="2">
-        <v>46146.38541666666</v>
+        <v>46148.38541666666</v>
       </c>
       <c r="B38">
         <v>0</v>
@@ -690,7 +690,7 @@
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="2">
-        <v>46146.39583333334</v>
+        <v>46148.39583333334</v>
       </c>
       <c r="B39">
         <v>0</v>
@@ -698,7 +698,7 @@
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="2">
-        <v>46146.40625</v>
+        <v>46148.40625</v>
       </c>
       <c r="B40">
         <v>0</v>
@@ -706,7 +706,7 @@
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="2">
-        <v>46146.41666666666</v>
+        <v>46148.41666666666</v>
       </c>
       <c r="B41">
         <v>0</v>
@@ -714,7 +714,7 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2">
-        <v>46146.42708333334</v>
+        <v>46148.42708333334</v>
       </c>
       <c r="B42">
         <v>0</v>
@@ -722,7 +722,7 @@
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="2">
-        <v>46146.4375</v>
+        <v>46148.4375</v>
       </c>
       <c r="B43">
         <v>0</v>
@@ -730,7 +730,7 @@
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="2">
-        <v>46146.44791666666</v>
+        <v>46148.44791666666</v>
       </c>
       <c r="B44">
         <v>0</v>
@@ -738,7 +738,7 @@
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="2">
-        <v>46146.45833333334</v>
+        <v>46148.45833333334</v>
       </c>
       <c r="B45">
         <v>0</v>
@@ -746,7 +746,7 @@
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="2">
-        <v>46146.46875</v>
+        <v>46148.46875</v>
       </c>
       <c r="B46">
         <v>0</v>
@@ -754,7 +754,7 @@
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="2">
-        <v>46146.47916666666</v>
+        <v>46148.47916666666</v>
       </c>
       <c r="B47">
         <v>0</v>
@@ -762,7 +762,7 @@
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="2">
-        <v>46146.48958333334</v>
+        <v>46148.48958333334</v>
       </c>
       <c r="B48">
         <v>0</v>
@@ -770,7 +770,7 @@
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="2">
-        <v>46146.5</v>
+        <v>46148.5</v>
       </c>
       <c r="B49">
         <v>0</v>
@@ -778,7 +778,7 @@
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="2">
-        <v>46146.51041666666</v>
+        <v>46148.51041666666</v>
       </c>
       <c r="B50">
         <v>0</v>
@@ -786,7 +786,7 @@
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="2">
-        <v>46146.52083333334</v>
+        <v>46148.52083333334</v>
       </c>
       <c r="B51">
         <v>0</v>
@@ -794,7 +794,7 @@
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="2">
-        <v>46146.53125</v>
+        <v>46148.53125</v>
       </c>
       <c r="B52">
         <v>0</v>
@@ -802,7 +802,7 @@
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="2">
-        <v>46146.54166666666</v>
+        <v>46148.54166666666</v>
       </c>
       <c r="B53">
         <v>0</v>
@@ -810,7 +810,7 @@
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="2">
-        <v>46146.55208333334</v>
+        <v>46148.55208333334</v>
       </c>
       <c r="B54">
         <v>0</v>
@@ -818,7 +818,7 @@
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="2">
-        <v>46146.5625</v>
+        <v>46148.5625</v>
       </c>
       <c r="B55">
         <v>0</v>
@@ -826,7 +826,7 @@
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="2">
-        <v>46146.57291666666</v>
+        <v>46148.57291666666</v>
       </c>
       <c r="B56">
         <v>0</v>
@@ -834,7 +834,7 @@
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="2">
-        <v>46146.58333333334</v>
+        <v>46148.58333333334</v>
       </c>
       <c r="B57">
         <v>0</v>
@@ -842,7 +842,7 @@
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="2">
-        <v>46146.59375</v>
+        <v>46148.59375</v>
       </c>
       <c r="B58">
         <v>0</v>
@@ -850,7 +850,7 @@
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="2">
-        <v>46146.60416666666</v>
+        <v>46148.60416666666</v>
       </c>
       <c r="B59">
         <v>0</v>
@@ -858,7 +858,7 @@
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="2">
-        <v>46146.61458333334</v>
+        <v>46148.61458333334</v>
       </c>
       <c r="B60">
         <v>0</v>
@@ -866,7 +866,7 @@
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="2">
-        <v>46146.625</v>
+        <v>46148.625</v>
       </c>
       <c r="B61">
         <v>0</v>
@@ -874,7 +874,7 @@
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="2">
-        <v>46146.63541666666</v>
+        <v>46148.63541666666</v>
       </c>
       <c r="B62">
         <v>0</v>
@@ -882,7 +882,7 @@
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="2">
-        <v>46146.64583333334</v>
+        <v>46148.64583333334</v>
       </c>
       <c r="B63">
         <v>0</v>
@@ -890,7 +890,7 @@
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="2">
-        <v>46146.65625</v>
+        <v>46148.65625</v>
       </c>
       <c r="B64">
         <v>0</v>
@@ -898,7 +898,7 @@
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="2">
-        <v>46146.66666666666</v>
+        <v>46148.66666666666</v>
       </c>
       <c r="B65">
         <v>0</v>
@@ -906,7 +906,7 @@
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="2">
-        <v>46146.67708333334</v>
+        <v>46148.67708333334</v>
       </c>
       <c r="B66">
         <v>0</v>
@@ -914,7 +914,7 @@
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="2">
-        <v>46146.6875</v>
+        <v>46148.6875</v>
       </c>
       <c r="B67">
         <v>0</v>
@@ -922,7 +922,7 @@
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="2">
-        <v>46146.69791666666</v>
+        <v>46148.69791666666</v>
       </c>
       <c r="B68">
         <v>0</v>
@@ -930,7 +930,7 @@
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="2">
-        <v>46146.70833333334</v>
+        <v>46148.70833333334</v>
       </c>
       <c r="B69">
         <v>0</v>
@@ -938,7 +938,7 @@
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="2">
-        <v>46146.71875</v>
+        <v>46148.71875</v>
       </c>
       <c r="B70">
         <v>0</v>
@@ -946,7 +946,7 @@
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="2">
-        <v>46146.72916666666</v>
+        <v>46148.72916666666</v>
       </c>
       <c r="B71">
         <v>0</v>
@@ -954,7 +954,7 @@
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="2">
-        <v>46146.73958333334</v>
+        <v>46148.73958333334</v>
       </c>
       <c r="B72">
         <v>0</v>
@@ -962,7 +962,7 @@
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="2">
-        <v>46146.75</v>
+        <v>46148.75</v>
       </c>
       <c r="B73">
         <v>0</v>
@@ -970,7 +970,7 @@
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="2">
-        <v>46146.76041666666</v>
+        <v>46148.76041666666</v>
       </c>
       <c r="B74">
         <v>0</v>
@@ -978,7 +978,7 @@
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="2">
-        <v>46146.77083333334</v>
+        <v>46148.77083333334</v>
       </c>
       <c r="B75">
         <v>0</v>
@@ -986,7 +986,7 @@
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="2">
-        <v>46146.78125</v>
+        <v>46148.78125</v>
       </c>
       <c r="B76">
         <v>0</v>
@@ -994,7 +994,7 @@
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="2">
-        <v>46146.79166666666</v>
+        <v>46148.79166666666</v>
       </c>
       <c r="B77">
         <v>0</v>
@@ -1002,7 +1002,7 @@
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="2">
-        <v>46146.80208333334</v>
+        <v>46148.80208333334</v>
       </c>
       <c r="B78">
         <v>0</v>
@@ -1010,7 +1010,7 @@
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="2">
-        <v>46146.8125</v>
+        <v>46148.8125</v>
       </c>
       <c r="B79">
         <v>0</v>
@@ -1018,7 +1018,7 @@
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="2">
-        <v>46146.82291666666</v>
+        <v>46148.82291666666</v>
       </c>
       <c r="B80">
         <v>0</v>
@@ -1026,7 +1026,7 @@
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="2">
-        <v>46146.83333333334</v>
+        <v>46148.83333333334</v>
       </c>
       <c r="B81">
         <v>0</v>
@@ -1034,7 +1034,7 @@
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="2">
-        <v>46146.84375</v>
+        <v>46148.84375</v>
       </c>
       <c r="B82">
         <v>0</v>
@@ -1042,7 +1042,7 @@
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="2">
-        <v>46146.85416666666</v>
+        <v>46148.85416666666</v>
       </c>
       <c r="B83">
         <v>0</v>
@@ -1050,7 +1050,7 @@
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="2">
-        <v>46146.86458333334</v>
+        <v>46148.86458333334</v>
       </c>
       <c r="B84">
         <v>0</v>
@@ -1058,7 +1058,7 @@
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="2">
-        <v>46146.875</v>
+        <v>46148.875</v>
       </c>
       <c r="B85">
         <v>0</v>
@@ -1066,7 +1066,7 @@
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="2">
-        <v>46146.88541666666</v>
+        <v>46148.88541666666</v>
       </c>
       <c r="B86">
         <v>0</v>
@@ -1074,7 +1074,7 @@
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="2">
-        <v>46146.89583333334</v>
+        <v>46148.89583333334</v>
       </c>
       <c r="B87">
         <v>0</v>
@@ -1082,7 +1082,7 @@
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="2">
-        <v>46146.90625</v>
+        <v>46148.90625</v>
       </c>
       <c r="B88">
         <v>0</v>
@@ -1090,7 +1090,7 @@
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="2">
-        <v>46146.91666666666</v>
+        <v>46148.91666666666</v>
       </c>
       <c r="B89">
         <v>0</v>
@@ -1098,7 +1098,7 @@
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="2">
-        <v>46146.92708333334</v>
+        <v>46148.92708333334</v>
       </c>
       <c r="B90">
         <v>0</v>
@@ -1106,7 +1106,7 @@
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="2">
-        <v>46146.9375</v>
+        <v>46148.9375</v>
       </c>
       <c r="B91">
         <v>0</v>
@@ -1114,7 +1114,7 @@
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="2">
-        <v>46146.94791666666</v>
+        <v>46148.94791666666</v>
       </c>
       <c r="B92">
         <v>0</v>
@@ -1122,7 +1122,7 @@
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="2">
-        <v>46146.95833333334</v>
+        <v>46148.95833333334</v>
       </c>
       <c r="B93">
         <v>0</v>
@@ -1130,7 +1130,7 @@
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="2">
-        <v>46146.96875</v>
+        <v>46148.96875</v>
       </c>
       <c r="B94">
         <v>0</v>
@@ -1138,7 +1138,7 @@
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="2">
-        <v>46146.97916666666</v>
+        <v>46148.97916666666</v>
       </c>
       <c r="B95">
         <v>0</v>
@@ -1146,7 +1146,7 @@
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="2">
-        <v>46146.98958333334</v>
+        <v>46148.98958333334</v>
       </c>
       <c r="B96">
         <v>0</v>
@@ -1154,7 +1154,7 @@
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="2">
-        <v>46147</v>
+        <v>46149</v>
       </c>
       <c r="B97">
         <v>0</v>

</xml_diff>